<commit_message>
[05/10] Mestra v4.3.5: Origem R70/R72 corrigida; venda L1623-T 05/10 lancada (linha 81); totais 31.651,40 / 8.073,60
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" tabRatio="500" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" tabRatio="500" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="LEIA-ME" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2049" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2052" uniqueCount="583">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -2044,7 +2044,21 @@
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -20161,7 +20175,7 @@
       </c>
       <c r="Q70" s="19"/>
       <c r="R70" s="19" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="S70" t="s">
         <v>558</v>
@@ -20295,7 +20309,7 @@
       </c>
       <c r="Q72" s="19"/>
       <c r="R72" s="19" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="S72" t="s">
         <v>558</v>
@@ -20815,57 +20829,70 @@
         <v>558</v>
       </c>
     </row>
-    <row r="81" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="32"/>
-      <c r="B81" s="19"/>
-      <c r="C81" s="19"/>
-      <c r="D81" s="19"/>
-      <c r="E81" s="20" t="str">
+    <row r="81" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="32">
+        <v>46300</v>
+      </c>
+      <c r="B81" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C81" s="19">
+        <v>1</v>
+      </c>
+      <c r="D81" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="E81" s="20">
         <f>IF($B81="","",INDEX(Simulador!$D$7:$D$232,MATCH($B81,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>123.93</v>
       </c>
       <c r="F81" s="20"/>
-      <c r="G81" s="13" t="str">
+      <c r="G81" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>123.93</v>
       </c>
       <c r="H81" s="8" t="str">
         <f>IF($B81="","",INDEX(Simulador!$B$7:$B$232,MATCH($B81,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I81" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I81" s="13">
         <f>IF(OR(H81="",$D81=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D81,Ref_Frete!$A$2:$A$54,0),IF(H81="Pequenos",2,IF(H81="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J81" s="20"/>
-      <c r="K81" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J81" s="20">
+        <v>16.36</v>
+      </c>
+      <c r="K81" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L81" s="13" t="str">
+        <v>20.09</v>
+      </c>
+      <c r="L81" s="13">
         <f>IF(OR($B81="",$C81=""),"",$C81*INDEX(Simulador!$F$7:$F$232,MATCH($B81,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M81" s="13" t="str">
+        <v>59.8</v>
+      </c>
+      <c r="M81" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N81" s="35" t="str">
+        <v>12.393000000000001</v>
+      </c>
+      <c r="N81" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O81" s="12" t="str">
+        <v>40.187000000000026</v>
+      </c>
+      <c r="O81" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.32427176631969679</v>
       </c>
       <c r="P81" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q81" s="19"/>
       <c r="R81" s="19"/>
-    </row>
-    <row r="82" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S81" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="82" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="32"/>
       <c r="B82" s="19"/>
       <c r="C82" s="19"/>
@@ -20915,7 +20942,7 @@
       <c r="Q82" s="19"/>
       <c r="R82" s="19"/>
     </row>
-    <row r="83" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="32"/>
       <c r="B83" s="19"/>
       <c r="C83" s="19"/>
@@ -20965,7 +20992,7 @@
       <c r="Q83" s="19"/>
       <c r="R83" s="19"/>
     </row>
-    <row r="84" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="32"/>
       <c r="B84" s="19"/>
       <c r="C84" s="19"/>
@@ -21015,7 +21042,7 @@
       <c r="Q84" s="19"/>
       <c r="R84" s="19"/>
     </row>
-    <row r="85" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="32"/>
       <c r="B85" s="19"/>
       <c r="C85" s="19"/>
@@ -21065,7 +21092,7 @@
       <c r="Q85" s="19"/>
       <c r="R85" s="19"/>
     </row>
-    <row r="86" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="32"/>
       <c r="B86" s="19"/>
       <c r="C86" s="19"/>
@@ -21115,7 +21142,7 @@
       <c r="Q86" s="19"/>
       <c r="R86" s="19"/>
     </row>
-    <row r="87" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="32"/>
       <c r="B87" s="19"/>
       <c r="C87" s="19"/>
@@ -21165,7 +21192,7 @@
       <c r="Q87" s="19"/>
       <c r="R87" s="19"/>
     </row>
-    <row r="88" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="32"/>
       <c r="B88" s="19"/>
       <c r="C88" s="19"/>
@@ -21215,7 +21242,7 @@
       <c r="Q88" s="19"/>
       <c r="R88" s="19"/>
     </row>
-    <row r="89" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="32"/>
       <c r="B89" s="19"/>
       <c r="C89" s="19"/>
@@ -21265,7 +21292,7 @@
       <c r="Q89" s="19"/>
       <c r="R89" s="19"/>
     </row>
-    <row r="90" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="32"/>
       <c r="B90" s="19"/>
       <c r="C90" s="19"/>
@@ -21315,7 +21342,7 @@
       <c r="Q90" s="19"/>
       <c r="R90" s="19"/>
     </row>
-    <row r="91" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="32"/>
       <c r="B91" s="19"/>
       <c r="C91" s="19"/>
@@ -21365,7 +21392,7 @@
       <c r="Q91" s="19"/>
       <c r="R91" s="19"/>
     </row>
-    <row r="92" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="32"/>
       <c r="B92" s="19"/>
       <c r="C92" s="19"/>
@@ -21415,7 +21442,7 @@
       <c r="Q92" s="19"/>
       <c r="R92" s="19"/>
     </row>
-    <row r="93" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="32"/>
       <c r="B93" s="19"/>
       <c r="C93" s="19"/>
@@ -21465,7 +21492,7 @@
       <c r="Q93" s="19"/>
       <c r="R93" s="19"/>
     </row>
-    <row r="94" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="32"/>
       <c r="B94" s="19"/>
       <c r="C94" s="19"/>
@@ -21515,7 +21542,7 @@
       <c r="Q94" s="19"/>
       <c r="R94" s="19"/>
     </row>
-    <row r="95" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="32"/>
       <c r="B95" s="19"/>
       <c r="C95" s="19"/>
@@ -21565,7 +21592,7 @@
       <c r="Q95" s="19"/>
       <c r="R95" s="19"/>
     </row>
-    <row r="96" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="32"/>
       <c r="B96" s="19"/>
       <c r="C96" s="19"/>
@@ -22171,38 +22198,38 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>31527.470000000016</v>
+        <v>31651.400000000016</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>4803.1600000000026</v>
+        <v>4823.2500000000027</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>16468.72</v>
+        <v>16528.52</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>3152.7469999999998</v>
+        <v>3165.14</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>8033.4130000000005</v>
+        <v>8073.6</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25480677643972055</v>
+        <v>0.25507876428846737</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S80">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+  <conditionalFormatting sqref="S6:S81">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"VÁLIDO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[08/10] Mestra: 4 vendas novas na semana do evento, todas fora das promocoes; L2460-CZ 1a venda — totais 32.484,66 / 8.319,10
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2052" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2064" uniqueCount="583">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -2044,21 +2044,7 @@
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -20893,204 +20879,256 @@
       </c>
     </row>
     <row r="82" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="32"/>
-      <c r="B82" s="19"/>
-      <c r="C82" s="19"/>
-      <c r="D82" s="19"/>
-      <c r="E82" s="20" t="str">
+      <c r="A82" s="32">
+        <v>46300</v>
+      </c>
+      <c r="B82" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C82" s="19">
+        <v>2</v>
+      </c>
+      <c r="D82" s="19" t="s">
+        <v>405</v>
+      </c>
+      <c r="E82" s="20">
         <f>IF($B82="","",INDEX(Simulador!$D$7:$D$232,MATCH($B82,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>132.9</v>
       </c>
       <c r="F82" s="20"/>
-      <c r="G82" s="13" t="str">
+      <c r="G82" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>265.8</v>
       </c>
       <c r="H82" s="8" t="str">
         <f>IF($B82="","",INDEX(Simulador!$B$7:$B$232,MATCH($B82,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I82" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I82" s="13">
         <f>IF(OR(H82="",$D82=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D82,Ref_Frete!$A$2:$A$54,0),IF(H82="Pequenos",2,IF(H82="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J82" s="20"/>
-      <c r="K82" s="20" t="str">
+        <v>29.9</v>
+      </c>
+      <c r="J82" s="20">
+        <v>26.11</v>
+      </c>
+      <c r="K82" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L82" s="13" t="str">
+        <v>39.92</v>
+      </c>
+      <c r="L82" s="13">
         <f>IF(OR($B82="",$C82=""),"",$C82*INDEX(Simulador!$F$7:$F$232,MATCH($B82,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M82" s="13" t="str">
+        <v>126.22</v>
+      </c>
+      <c r="M82" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N82" s="35" t="str">
+        <v>26.580000000000002</v>
+      </c>
+      <c r="N82" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O82" s="12" t="str">
+        <v>76.869999999999962</v>
+      </c>
+      <c r="O82" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.28920240782543249</v>
       </c>
       <c r="P82" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q82" s="19"/>
       <c r="R82" s="19"/>
+      <c r="S82" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="83" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="32"/>
-      <c r="B83" s="19"/>
-      <c r="C83" s="19"/>
-      <c r="D83" s="19"/>
-      <c r="E83" s="20" t="str">
+      <c r="A83" s="32">
+        <v>46302</v>
+      </c>
+      <c r="B83" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C83" s="19">
+        <v>1</v>
+      </c>
+      <c r="D83" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E83" s="20">
         <f>IF($B83="","",INDEX(Simulador!$D$7:$D$232,MATCH($B83,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>116</v>
       </c>
       <c r="F83" s="20"/>
-      <c r="G83" s="13" t="str">
+      <c r="G83" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>116</v>
       </c>
       <c r="H83" s="8" t="str">
         <f>IF($B83="","",INDEX(Simulador!$B$7:$B$232,MATCH($B83,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I83" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I83" s="13">
         <f>IF(OR(H83="",$D83=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D83,Ref_Frete!$A$2:$A$54,0),IF(H83="Pequenos",2,IF(H83="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J83" s="20"/>
-      <c r="K83" s="20" t="str">
+        <v>16.899999999999999</v>
+      </c>
+      <c r="J83" s="20">
+        <v>18</v>
+      </c>
+      <c r="K83" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L83" s="13" t="str">
+        <v>17.940000000000001</v>
+      </c>
+      <c r="L83" s="13">
         <f>IF(OR($B83="",$C83=""),"",$C83*INDEX(Simulador!$F$7:$F$232,MATCH($B83,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M83" s="13" t="str">
+        <v>54.47</v>
+      </c>
+      <c r="M83" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N83" s="35" t="str">
+        <v>11.600000000000001</v>
+      </c>
+      <c r="N83" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O83" s="12" t="str">
+        <v>30.890000000000008</v>
+      </c>
+      <c r="O83" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.26629310344827595</v>
       </c>
       <c r="P83" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q83" s="19"/>
       <c r="R83" s="19"/>
+      <c r="S83" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="84" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="32"/>
-      <c r="B84" s="19"/>
-      <c r="C84" s="19"/>
-      <c r="D84" s="19"/>
-      <c r="E84" s="20" t="str">
+      <c r="A84" s="32">
+        <v>46303</v>
+      </c>
+      <c r="B84" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C84" s="19">
+        <v>1</v>
+      </c>
+      <c r="D84" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="E84" s="20">
         <f>IF($B84="","",INDEX(Simulador!$D$7:$D$232,MATCH($B84,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>132.9</v>
       </c>
       <c r="F84" s="20"/>
-      <c r="G84" s="13" t="str">
+      <c r="G84" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>132.9</v>
       </c>
       <c r="H84" s="8" t="str">
         <f>IF($B84="","",INDEX(Simulador!$B$7:$B$232,MATCH($B84,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I84" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I84" s="13">
         <f>IF(OR(H84="",$D84=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D84,Ref_Frete!$A$2:$A$54,0),IF(H84="Pequenos",2,IF(H84="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J84" s="20"/>
-      <c r="K84" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J84" s="20">
+        <v>16.36</v>
+      </c>
+      <c r="K84" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L84" s="13" t="str">
+        <v>21.3</v>
+      </c>
+      <c r="L84" s="13">
         <f>IF(OR($B84="",$C84=""),"",$C84*INDEX(Simulador!$F$7:$F$232,MATCH($B84,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M84" s="13" t="str">
+        <v>63.11</v>
+      </c>
+      <c r="M84" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N84" s="35" t="str">
+        <v>13.290000000000001</v>
+      </c>
+      <c r="N84" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O84" s="12" t="str">
+        <v>43.74</v>
+      </c>
+      <c r="O84" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.32911963882618511</v>
       </c>
       <c r="P84" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q84" s="19"/>
       <c r="R84" s="19"/>
+      <c r="S84" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="85" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="32"/>
-      <c r="B85" s="19"/>
-      <c r="C85" s="19"/>
-      <c r="D85" s="19"/>
-      <c r="E85" s="20" t="str">
+      <c r="A85" s="32">
+        <v>46303</v>
+      </c>
+      <c r="B85" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="C85" s="19">
+        <v>1</v>
+      </c>
+      <c r="D85" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="E85" s="20">
         <f>IF($B85="","",INDEX(Simulador!$D$7:$D$232,MATCH($B85,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>318.56</v>
       </c>
       <c r="F85" s="20"/>
-      <c r="G85" s="13" t="str">
+      <c r="G85" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>318.56</v>
       </c>
       <c r="H85" s="8" t="str">
         <f>IF($B85="","",INDEX(Simulador!$B$7:$B$232,MATCH($B85,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I85" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I85" s="13">
         <f>IF(OR(H85="",$D85=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D85,Ref_Frete!$A$2:$A$54,0),IF(H85="Pequenos",2,IF(H85="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J85" s="20"/>
-      <c r="K85" s="20" t="str">
+        <v>34.9</v>
+      </c>
+      <c r="J85" s="20">
+        <v>20.88</v>
+      </c>
+      <c r="K85" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L85" s="13" t="str">
+        <v>47.72</v>
+      </c>
+      <c r="L85" s="13">
         <f>IF(OR($B85="",$C85=""),"",$C85*INDEX(Simulador!$F$7:$F$232,MATCH($B85,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M85" s="13" t="str">
+        <v>159</v>
+      </c>
+      <c r="M85" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N85" s="35" t="str">
+        <v>31.856000000000002</v>
+      </c>
+      <c r="N85" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O85" s="12" t="str">
+        <v>94.004000000000019</v>
+      </c>
+      <c r="O85" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.29509040683073839</v>
       </c>
       <c r="P85" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q85" s="19"/>
       <c r="R85" s="19"/>
+      <c r="S85" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="86" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="32"/>
@@ -22198,38 +22236,38 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>31651.400000000016</v>
+        <v>32484.660000000018</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>4823.2500000000027</v>
+        <v>4950.1300000000028</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>16528.52</v>
+        <v>16931.320000000003</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>3165.14</v>
+        <v>3248.4659999999999</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>8073.6</v>
+        <v>8319.1040000000012</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25507876428846737</v>
+        <v>0.256093306810045</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S81">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+  <conditionalFormatting sqref="S6:S85">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"VÁLIDO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[13/10] Mestra: semana do Prime Day no Registro — 12 pedidos / 20 un / R$ 3.159,32, zero vendas a preco promocional nos 14 SKUs; 3 primeiras vendas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2064" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2079" uniqueCount="583">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -2044,7 +2044,21 @@
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -21131,351 +21145,428 @@
       </c>
     </row>
     <row r="86" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="32"/>
-      <c r="B86" s="19"/>
-      <c r="C86" s="19"/>
-      <c r="D86" s="19"/>
-      <c r="E86" s="20" t="str">
+      <c r="A86" s="32">
+        <v>46304</v>
+      </c>
+      <c r="B86" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C86" s="19">
+        <v>1</v>
+      </c>
+      <c r="D86" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="E86" s="20">
         <f>IF($B86="","",INDEX(Simulador!$D$7:$D$232,MATCH($B86,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>109.9</v>
       </c>
       <c r="F86" s="20"/>
-      <c r="G86" s="13" t="str">
+      <c r="G86" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>109.9</v>
       </c>
       <c r="H86" s="8" t="str">
         <f>IF($B86="","",INDEX(Simulador!$B$7:$B$232,MATCH($B86,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I86" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I86" s="13">
         <f>IF(OR(H86="",$D86=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D86,Ref_Frete!$A$2:$A$54,0),IF(H86="Pequenos",2,IF(H86="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J86" s="20"/>
-      <c r="K86" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J86" s="20">
+        <v>16.36</v>
+      </c>
+      <c r="K86" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L86" s="13" t="str">
+        <v>18.2</v>
+      </c>
+      <c r="L86" s="13">
         <f>IF(OR($B86="",$C86=""),"",$C86*INDEX(Simulador!$F$7:$F$232,MATCH($B86,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M86" s="13" t="str">
+        <v>49.15</v>
+      </c>
+      <c r="M86" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N86" s="35" t="str">
+        <v>10.990000000000002</v>
+      </c>
+      <c r="N86" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O86" s="12" t="str">
+        <v>40.100000000000009</v>
+      </c>
+      <c r="O86" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.36487716105550505</v>
       </c>
       <c r="P86" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q86" s="19"/>
       <c r="R86" s="19"/>
+      <c r="S86" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="87" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="32"/>
-      <c r="B87" s="19"/>
-      <c r="C87" s="19"/>
-      <c r="D87" s="19"/>
-      <c r="E87" s="20" t="str">
+      <c r="A87" s="32">
+        <v>46305</v>
+      </c>
+      <c r="B87" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C87" s="19">
+        <v>1</v>
+      </c>
+      <c r="D87" s="19" t="s">
+        <v>406</v>
+      </c>
+      <c r="E87" s="20">
         <f>IF($B87="","",INDEX(Simulador!$D$7:$D$232,MATCH($B87,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>119.22</v>
       </c>
       <c r="F87" s="20"/>
-      <c r="G87" s="13" t="str">
+      <c r="G87" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>119.22</v>
       </c>
       <c r="H87" s="8" t="str">
         <f>IF($B87="","",INDEX(Simulador!$B$7:$B$232,MATCH($B87,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I87" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I87" s="13">
         <f>IF(OR(H87="",$D87=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D87,Ref_Frete!$A$2:$A$54,0),IF(H87="Pequenos",2,IF(H87="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J87" s="20"/>
-      <c r="K87" s="20" t="str">
+        <v>29.9</v>
+      </c>
+      <c r="J87" s="20">
+        <v>23.75</v>
+      </c>
+      <c r="K87" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L87" s="13" t="str">
+        <v>20.13</v>
+      </c>
+      <c r="L87" s="13">
         <f>IF(OR($B87="",$C87=""),"",$C87*INDEX(Simulador!$F$7:$F$232,MATCH($B87,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M87" s="13" t="str">
+        <v>55.49</v>
+      </c>
+      <c r="M87" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N87" s="35" t="str">
+        <v>11.922000000000001</v>
+      </c>
+      <c r="N87" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O87" s="12" t="str">
+        <v>37.828000000000003</v>
+      </c>
+      <c r="O87" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.31729575574568031</v>
       </c>
       <c r="P87" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q87" s="19"/>
       <c r="R87" s="19"/>
     </row>
     <row r="88" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="32"/>
-      <c r="B88" s="19"/>
-      <c r="C88" s="19"/>
-      <c r="D88" s="19"/>
-      <c r="E88" s="20" t="str">
+      <c r="A88" s="32">
+        <v>46305</v>
+      </c>
+      <c r="B88" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C88" s="19">
+        <v>2</v>
+      </c>
+      <c r="D88" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E88" s="20">
         <f>IF($B88="","",INDEX(Simulador!$D$7:$D$232,MATCH($B88,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>132.9</v>
       </c>
       <c r="F88" s="20"/>
-      <c r="G88" s="13" t="str">
+      <c r="G88" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>265.8</v>
       </c>
       <c r="H88" s="8" t="str">
         <f>IF($B88="","",INDEX(Simulador!$B$7:$B$232,MATCH($B88,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I88" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I88" s="13">
         <f>IF(OR(H88="",$D88=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D88,Ref_Frete!$A$2:$A$54,0),IF(H88="Pequenos",2,IF(H88="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J88" s="20"/>
-      <c r="K88" s="20" t="str">
+        <v>16.899999999999999</v>
+      </c>
+      <c r="J88" s="20">
+        <v>18</v>
+      </c>
+      <c r="K88" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L88" s="13" t="str">
+        <v>38.159999999999997</v>
+      </c>
+      <c r="L88" s="13">
         <f>IF(OR($B88="",$C88=""),"",$C88*INDEX(Simulador!$F$7:$F$232,MATCH($B88,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M88" s="13" t="str">
+        <v>126.22</v>
+      </c>
+      <c r="M88" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N88" s="35" t="str">
+        <v>26.580000000000002</v>
+      </c>
+      <c r="N88" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O88" s="12" t="str">
+        <v>73.739999999999995</v>
+      </c>
+      <c r="O88" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.27742663656884875</v>
       </c>
       <c r="P88" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q88" s="19"/>
       <c r="R88" s="19"/>
     </row>
     <row r="89" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="32"/>
-      <c r="B89" s="19"/>
-      <c r="C89" s="19"/>
-      <c r="D89" s="19"/>
-      <c r="E89" s="20" t="str">
+      <c r="A89" s="32">
+        <v>46306</v>
+      </c>
+      <c r="B89" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C89" s="19">
+        <v>1</v>
+      </c>
+      <c r="D89" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="E89" s="20">
         <f>IF($B89="","",INDEX(Simulador!$D$7:$D$232,MATCH($B89,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>616.17999999999995</v>
       </c>
       <c r="F89" s="20"/>
-      <c r="G89" s="13" t="str">
+      <c r="G89" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>616.17999999999995</v>
       </c>
       <c r="H89" s="8" t="str">
         <f>IF($B89="","",INDEX(Simulador!$B$7:$B$232,MATCH($B89,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I89" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I89" s="13">
         <f>IF(OR(H89="",$D89=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D89,Ref_Frete!$A$2:$A$54,0),IF(H89="Pequenos",2,IF(H89="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J89" s="20"/>
-      <c r="K89" s="20" t="str">
+        <v>59.9</v>
+      </c>
+      <c r="J89" s="20">
+        <v>58.1</v>
+      </c>
+      <c r="K89" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L89" s="13" t="str">
+        <v>91.27</v>
+      </c>
+      <c r="L89" s="13">
         <f>IF(OR($B89="",$C89=""),"",$C89*INDEX(Simulador!$F$7:$F$232,MATCH($B89,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M89" s="13" t="str">
+        <v>307.26</v>
+      </c>
+      <c r="M89" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N89" s="35" t="str">
+        <v>61.617999999999995</v>
+      </c>
+      <c r="N89" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O89" s="12" t="str">
+        <v>157.83199999999994</v>
+      </c>
+      <c r="O89" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.25614593138368652</v>
       </c>
       <c r="P89" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q89" s="19"/>
       <c r="R89" s="19"/>
     </row>
     <row r="90" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="32"/>
-      <c r="B90" s="19"/>
-      <c r="C90" s="19"/>
-      <c r="D90" s="19"/>
-      <c r="E90" s="20" t="str">
+      <c r="A90" s="32">
+        <v>46306</v>
+      </c>
+      <c r="B90" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="C90" s="19">
+        <v>5</v>
+      </c>
+      <c r="D90" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="E90" s="20">
         <f>IF($B90="","",INDEX(Simulador!$D$7:$D$232,MATCH($B90,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="F90" s="20"/>
-      <c r="G90" s="13" t="str">
+        <v>127.9</v>
+      </c>
+      <c r="F90" s="20">
+        <v>51.16</v>
+      </c>
+      <c r="G90" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>588.34</v>
       </c>
       <c r="H90" s="8" t="str">
         <f>IF($B90="","",INDEX(Simulador!$B$7:$B$232,MATCH($B90,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I90" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I90" s="13">
         <f>IF(OR(H90="",$D90=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D90,Ref_Frete!$A$2:$A$54,0),IF(H90="Pequenos",2,IF(H90="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J90" s="20"/>
-      <c r="K90" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J90" s="20">
+        <v>89.54</v>
+      </c>
+      <c r="K90" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L90" s="13" t="str">
+        <v>82.79</v>
+      </c>
+      <c r="L90" s="13">
         <f>IF(OR($B90="",$C90=""),"",$C90*INDEX(Simulador!$F$7:$F$232,MATCH($B90,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M90" s="13" t="str">
+        <v>301.05</v>
+      </c>
+      <c r="M90" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N90" s="35" t="str">
+        <v>58.834000000000003</v>
+      </c>
+      <c r="N90" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O90" s="12" t="str">
+        <v>81.02600000000001</v>
+      </c>
+      <c r="O90" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.13771968589591055</v>
       </c>
       <c r="P90" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ABAIXO DA META (10-15%)</v>
       </c>
       <c r="Q90" s="19"/>
       <c r="R90" s="19"/>
     </row>
     <row r="91" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="32"/>
-      <c r="B91" s="19"/>
-      <c r="C91" s="19"/>
-      <c r="D91" s="19"/>
-      <c r="E91" s="20" t="str">
+      <c r="A91" s="32">
+        <v>46306</v>
+      </c>
+      <c r="B91" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C91" s="19">
+        <v>3</v>
+      </c>
+      <c r="D91" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E91" s="20">
         <f>IF($B91="","",INDEX(Simulador!$D$7:$D$232,MATCH($B91,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="F91" s="20"/>
-      <c r="G91" s="13" t="str">
+        <v>132.9</v>
+      </c>
+      <c r="F91" s="20">
+        <v>19.940000000000001</v>
+      </c>
+      <c r="G91" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>378.76000000000005</v>
       </c>
       <c r="H91" s="8" t="str">
         <f>IF($B91="","",INDEX(Simulador!$B$7:$B$232,MATCH($B91,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I91" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I91" s="13">
         <f>IF(OR(H91="",$D91=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D91,Ref_Frete!$A$2:$A$54,0),IF(H91="Pequenos",2,IF(H91="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J91" s="20"/>
-      <c r="K91" s="20" t="str">
+        <v>16.899999999999999</v>
+      </c>
+      <c r="J91" s="20">
+        <v>24.39</v>
+      </c>
+      <c r="K91" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L91" s="13" t="str">
+        <v>53.41</v>
+      </c>
+      <c r="L91" s="13">
         <f>IF(OR($B91="",$C91=""),"",$C91*INDEX(Simulador!$F$7:$F$232,MATCH($B91,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M91" s="13" t="str">
+        <v>189.32999999999998</v>
+      </c>
+      <c r="M91" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N91" s="35" t="str">
+        <v>37.876000000000005</v>
+      </c>
+      <c r="N91" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O91" s="12" t="str">
+        <v>90.654000000000025</v>
+      </c>
+      <c r="O91" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.23934417573133387</v>
       </c>
       <c r="P91" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q91" s="19"/>
       <c r="R91" s="19"/>
     </row>
     <row r="92" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="32"/>
-      <c r="B92" s="19"/>
-      <c r="C92" s="19"/>
-      <c r="D92" s="19"/>
-      <c r="E92" s="20" t="str">
+      <c r="A92" s="32">
+        <v>46306</v>
+      </c>
+      <c r="B92" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C92" s="19">
+        <v>1</v>
+      </c>
+      <c r="D92" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="E92" s="20">
         <f>IF($B92="","",INDEX(Simulador!$D$7:$D$232,MATCH($B92,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>123.93</v>
       </c>
       <c r="F92" s="20"/>
-      <c r="G92" s="13" t="str">
+      <c r="G92" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>123.93</v>
       </c>
       <c r="H92" s="8" t="str">
         <f>IF($B92="","",INDEX(Simulador!$B$7:$B$232,MATCH($B92,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I92" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I92" s="13">
         <f>IF(OR(H92="",$D92=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D92,Ref_Frete!$A$2:$A$54,0),IF(H92="Pequenos",2,IF(H92="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J92" s="20"/>
-      <c r="K92" s="20" t="str">
+        <v>12.9</v>
+      </c>
+      <c r="J92" s="20">
+        <v>12.87</v>
+      </c>
+      <c r="K92" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L92" s="13" t="str">
+        <v>18.47</v>
+      </c>
+      <c r="L92" s="13">
         <f>IF(OR($B92="",$C92=""),"",$C92*INDEX(Simulador!$F$7:$F$232,MATCH($B92,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M92" s="13" t="str">
+        <v>59.8</v>
+      </c>
+      <c r="M92" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N92" s="35" t="str">
+        <v>12.393000000000001</v>
+      </c>
+      <c r="N92" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O92" s="12" t="str">
+        <v>33.297000000000011</v>
+      </c>
+      <c r="O92" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.26867586540789162</v>
       </c>
       <c r="P92" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q92" s="19"/>
       <c r="R92" s="19"/>
@@ -22236,38 +22327,38 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>32484.660000000018</v>
+        <v>34686.790000000023</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>4950.1300000000028</v>
+        <v>5272.5600000000031</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>16931.320000000003</v>
+        <v>18019.620000000006</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>3248.4659999999999</v>
+        <v>3468.6789999999996</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>8319.1040000000012</v>
+        <v>8833.5810000000019</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.256093306810045</v>
+        <v>0.25466700723820213</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S85">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+  <conditionalFormatting sqref="S6:S86">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"VÁLIDO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[13/10] Mestra: Origem 83-92 e STATUS 87-92 preenchidos conforme a semana 06-12/10
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2079" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2095" uniqueCount="583">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -21013,7 +21013,9 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q83" s="19"/>
-      <c r="R83" s="19"/>
+      <c r="R83" s="19" t="s">
+        <v>210</v>
+      </c>
       <c r="S83" t="s">
         <v>558</v>
       </c>
@@ -21076,7 +21078,9 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q84" s="19"/>
-      <c r="R84" s="19"/>
+      <c r="R84" s="19" t="s">
+        <v>210</v>
+      </c>
       <c r="S84" t="s">
         <v>558</v>
       </c>
@@ -21139,7 +21143,9 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q85" s="19"/>
-      <c r="R85" s="19"/>
+      <c r="R85" s="19" t="s">
+        <v>210</v>
+      </c>
       <c r="S85" t="s">
         <v>558</v>
       </c>
@@ -21202,7 +21208,9 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q86" s="19"/>
-      <c r="R86" s="19"/>
+      <c r="R86" s="19" t="s">
+        <v>210</v>
+      </c>
       <c r="S86" t="s">
         <v>558</v>
       </c>
@@ -21265,7 +21273,12 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q87" s="19"/>
-      <c r="R87" s="19"/>
+      <c r="R87" s="19" t="s">
+        <v>207</v>
+      </c>
+      <c r="S87" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="88" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="32">
@@ -21325,7 +21338,12 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q88" s="19"/>
-      <c r="R88" s="19"/>
+      <c r="R88" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="S88" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="89" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="32">
@@ -21385,7 +21403,12 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q89" s="19"/>
-      <c r="R89" s="19"/>
+      <c r="R89" s="19" t="s">
+        <v>207</v>
+      </c>
+      <c r="S89" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="90" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="32">
@@ -21447,7 +21470,12 @@
         <v>ABAIXO DA META (10-15%)</v>
       </c>
       <c r="Q90" s="19"/>
-      <c r="R90" s="19"/>
+      <c r="R90" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="S90" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="91" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="32">
@@ -21509,7 +21537,12 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q91" s="19"/>
-      <c r="R91" s="19"/>
+      <c r="R91" s="19" t="s">
+        <v>207</v>
+      </c>
+      <c r="S91" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="92" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="32">
@@ -21569,7 +21602,12 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q92" s="19"/>
-      <c r="R92" s="19"/>
+      <c r="R92" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="S92" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="93" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="32"/>
@@ -22354,7 +22392,7 @@
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S86">
+  <conditionalFormatting sqref="S6:S92">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>

</xml_diff>

<commit_message>
[O7 13/10] Mestra: correcoes R81 Ads, R82 Organico e desconto F89 (P3070 11/10) lancadas pelo LEO; ressalva de R$ 0,09 (92,34 vs 92,43) anotada
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2095" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2097" uniqueCount="583">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -2044,21 +2044,7 @@
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -20887,7 +20873,9 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q81" s="19"/>
-      <c r="R81" s="19"/>
+      <c r="R81" s="19" t="s">
+        <v>210</v>
+      </c>
       <c r="S81" t="s">
         <v>558</v>
       </c>
@@ -20950,7 +20938,9 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q82" s="19"/>
-      <c r="R82" s="19"/>
+      <c r="R82" s="19" t="s">
+        <v>207</v>
+      </c>
       <c r="S82" t="s">
         <v>558</v>
       </c>
@@ -21362,10 +21352,12 @@
         <f>IF($B89="","",INDEX(Simulador!$D$7:$D$232,MATCH($B89,Simulador!$A$7:$A$232,0)))</f>
         <v>616.17999999999995</v>
       </c>
-      <c r="F89" s="20"/>
+      <c r="F89" s="20">
+        <v>92.34</v>
+      </c>
       <c r="G89" s="13">
         <f t="shared" si="12"/>
-        <v>616.17999999999995</v>
+        <v>523.83999999999992</v>
       </c>
       <c r="H89" s="8" t="str">
         <f>IF($B89="","",INDEX(Simulador!$B$7:$B$232,MATCH($B89,Simulador!$A$7:$A$232,0)))</f>
@@ -21380,7 +21372,7 @@
       </c>
       <c r="K89" s="20">
         <f t="shared" si="17"/>
-        <v>91.27</v>
+        <v>78.8</v>
       </c>
       <c r="L89" s="13">
         <f>IF(OR($B89="",$C89=""),"",$C89*INDEX(Simulador!$F$7:$F$232,MATCH($B89,Simulador!$A$7:$A$232,0)))</f>
@@ -21388,19 +21380,19 @@
       </c>
       <c r="M89" s="13">
         <f t="shared" si="13"/>
-        <v>61.617999999999995</v>
+        <v>52.383999999999993</v>
       </c>
       <c r="N89" s="35">
         <f t="shared" si="14"/>
-        <v>157.83199999999994</v>
+        <v>87.195999999999884</v>
       </c>
       <c r="O89" s="12">
         <f t="shared" si="15"/>
-        <v>0.25614593138368652</v>
+        <v>0.16645540623091001</v>
       </c>
       <c r="P89" s="22" t="str">
         <f t="shared" si="16"/>
-        <v>ACIMA DA META (&gt;20%)</v>
+        <v>DENTRO DA META (15-20%)</v>
       </c>
       <c r="Q89" s="19"/>
       <c r="R89" s="19" t="s">
@@ -22365,11 +22357,11 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>34686.790000000023</v>
+        <v>34594.450000000019</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>5272.5600000000031</v>
+        <v>5260.0900000000029</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
@@ -22377,15 +22369,15 @@
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>3468.6789999999996</v>
+        <v>3459.4449999999997</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>8833.5810000000019</v>
+        <v>8762.9450000000015</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25466700723820213</v>
+        <v>0.25330493764173145</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -22393,10 +22385,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="S6:S92">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"VÁLIDO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[O7 13/10] conferencia 1 da execucao: 7 acoes conferidas por export/prints, 9 aguardando print, 6B ainda dinamica no export; Mestra F89 corrigida (92,43); Parametros s3 com valores pos-execucao conferidos
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -21353,11 +21353,11 @@
         <v>616.17999999999995</v>
       </c>
       <c r="F89" s="20">
-        <v>92.34</v>
+        <v>92.43</v>
       </c>
       <c r="G89" s="13">
         <f t="shared" si="12"/>
-        <v>523.83999999999992</v>
+        <v>523.75</v>
       </c>
       <c r="H89" s="8" t="str">
         <f>IF($B89="","",INDEX(Simulador!$B$7:$B$232,MATCH($B89,Simulador!$A$7:$A$232,0)))</f>
@@ -21372,7 +21372,7 @@
       </c>
       <c r="K89" s="20">
         <f t="shared" si="17"/>
-        <v>78.8</v>
+        <v>78.790000000000006</v>
       </c>
       <c r="L89" s="13">
         <f>IF(OR($B89="",$C89=""),"",$C89*INDEX(Simulador!$F$7:$F$232,MATCH($B89,Simulador!$A$7:$A$232,0)))</f>
@@ -21380,15 +21380,15 @@
       </c>
       <c r="M89" s="13">
         <f t="shared" si="13"/>
-        <v>52.383999999999993</v>
+        <v>52.375</v>
       </c>
       <c r="N89" s="35">
         <f t="shared" si="14"/>
-        <v>87.195999999999884</v>
+        <v>87.124999999999943</v>
       </c>
       <c r="O89" s="12">
         <f t="shared" si="15"/>
-        <v>0.16645540623091001</v>
+        <v>0.16634844868735071</v>
       </c>
       <c r="P89" s="22" t="str">
         <f t="shared" si="16"/>
@@ -22357,11 +22357,11 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>34594.450000000019</v>
+        <v>34594.360000000022</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>5260.0900000000029</v>
+        <v>5260.0800000000027</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
@@ -22369,15 +22369,15 @@
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>3459.4449999999997</v>
+        <v>3459.4359999999997</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>8762.9450000000015</v>
+        <v>8762.8740000000016</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25330493764173145</v>
+        <v>0.25330354427715951</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
[15/10] Mestra: venda de 13/10 (L1618-B, DF) lancada pelo LEO na linha 93; Origem/STATUS pendentes; ressalva de frete cobrado x real anotada
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2097" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2099" uniqueCount="583">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -21602,51 +21602,61 @@
       </c>
     </row>
     <row r="93" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="32"/>
-      <c r="B93" s="19"/>
-      <c r="C93" s="19"/>
-      <c r="D93" s="19"/>
-      <c r="E93" s="20" t="str">
+      <c r="A93" s="32">
+        <v>46308</v>
+      </c>
+      <c r="B93" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="C93" s="19">
+        <v>1</v>
+      </c>
+      <c r="D93" s="19" t="s">
+        <v>206</v>
+      </c>
+      <c r="E93" s="20">
         <f>IF($B93="","",INDEX(Simulador!$D$7:$D$232,MATCH($B93,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>129.9</v>
       </c>
       <c r="F93" s="20"/>
-      <c r="G93" s="13" t="str">
+      <c r="G93" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>129.9</v>
       </c>
       <c r="H93" s="8" t="str">
         <f>IF($B93="","",INDEX(Simulador!$B$7:$B$232,MATCH($B93,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I93" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I93" s="13">
         <f>IF(OR(H93="",$D93=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D93,Ref_Frete!$A$2:$A$54,0),IF(H93="Pequenos",2,IF(H93="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J93" s="20"/>
-      <c r="K93" s="20" t="str">
+        <v>52</v>
+      </c>
+      <c r="J93" s="20">
+        <v>16.04</v>
+      </c>
+      <c r="K93" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L93" s="13" t="str">
+        <v>24.56</v>
+      </c>
+      <c r="L93" s="13">
         <f>IF(OR($B93="",$C93=""),"",$C93*INDEX(Simulador!$F$7:$F$232,MATCH($B93,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M93" s="13" t="str">
+        <v>60.62</v>
+      </c>
+      <c r="M93" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N93" s="35" t="str">
+        <v>12.990000000000002</v>
+      </c>
+      <c r="N93" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O93" s="12" t="str">
+        <v>67.69</v>
+      </c>
+      <c r="O93" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.52109314857582756</v>
       </c>
       <c r="P93" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q93" s="19"/>
       <c r="R93" s="19"/>
@@ -22357,27 +22367,27 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>34594.360000000022</v>
+        <v>34724.260000000024</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>5260.0800000000027</v>
+        <v>5284.6400000000031</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>18019.620000000006</v>
+        <v>18080.240000000005</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>3459.4359999999997</v>
+        <v>3472.4259999999995</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>8762.8740000000016</v>
+        <v>8830.5640000000021</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25330354427715951</v>
+        <v>0.25430531852946603</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
[16/10] Mestra: venda de 15/10 (P3070, PR Interior) lancada na linha 94 e STATUS VALIDO em 93/94; Origem pendente do export Ads
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2099" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2103" uniqueCount="583">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -21660,56 +21660,72 @@
       </c>
       <c r="Q93" s="19"/>
       <c r="R93" s="19"/>
+      <c r="S93" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="94" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="32"/>
-      <c r="B94" s="19"/>
-      <c r="C94" s="19"/>
-      <c r="D94" s="19"/>
-      <c r="E94" s="20" t="str">
+      <c r="A94" s="32">
+        <v>46310</v>
+      </c>
+      <c r="B94" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C94" s="19">
+        <v>1</v>
+      </c>
+      <c r="D94" s="19" t="s">
+        <v>405</v>
+      </c>
+      <c r="E94" s="20">
         <f>IF($B94="","",INDEX(Simulador!$D$7:$D$232,MATCH($B94,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>616.17999999999995</v>
       </c>
       <c r="F94" s="20"/>
-      <c r="G94" s="13" t="str">
+      <c r="G94" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>616.17999999999995</v>
       </c>
       <c r="H94" s="8" t="str">
         <f>IF($B94="","",INDEX(Simulador!$B$7:$B$232,MATCH($B94,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I94" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I94" s="13">
         <f>IF(OR(H94="",$D94=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D94,Ref_Frete!$A$2:$A$54,0),IF(H94="Pequenos",2,IF(H94="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J94" s="20"/>
-      <c r="K94" s="20" t="str">
+        <v>69.900000000000006</v>
+      </c>
+      <c r="J94" s="20">
+        <v>63.46</v>
+      </c>
+      <c r="K94" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L94" s="13" t="str">
+        <v>92.62</v>
+      </c>
+      <c r="L94" s="13">
         <f>IF(OR($B94="",$C94=""),"",$C94*INDEX(Simulador!$F$7:$F$232,MATCH($B94,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M94" s="13" t="str">
+        <v>307.26</v>
+      </c>
+      <c r="M94" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N94" s="35" t="str">
+        <v>61.617999999999995</v>
+      </c>
+      <c r="N94" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O94" s="12" t="str">
+        <v>161.1219999999999</v>
+      </c>
+      <c r="O94" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.26148528027524409</v>
       </c>
       <c r="P94" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q94" s="19"/>
       <c r="R94" s="19"/>
+      <c r="S94" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="95" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="32"/>
@@ -22367,34 +22383,34 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>34724.260000000024</v>
+        <v>35340.440000000024</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>5284.6400000000031</v>
+        <v>5377.2600000000029</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>18080.240000000005</v>
+        <v>18387.500000000004</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>3472.4259999999995</v>
+        <v>3534.0439999999994</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>8830.5640000000021</v>
+        <v>8991.6860000000015</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25430531852946603</v>
+        <v>0.25443050510972687</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S92">
+  <conditionalFormatting sqref="S6:S94">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>

</xml_diff>

<commit_message>
[19/10] monitoramento semanal 13-19/10: 125 cli / R$ 99,02 / 1 compra / ACOS 76%; entrega -34% e conversao da Geral 0,9%; NAO DECIDIR AINDA com checkpoint 22/10; Mestra linha 95; linha 17 do Controle proposta
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2103" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2105" uniqueCount="583">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -21728,51 +21728,61 @@
       </c>
     </row>
     <row r="95" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="32"/>
-      <c r="B95" s="19"/>
-      <c r="C95" s="19"/>
-      <c r="D95" s="19"/>
-      <c r="E95" s="20" t="str">
+      <c r="A95" s="32">
+        <v>46314</v>
+      </c>
+      <c r="B95" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C95" s="19">
+        <v>1</v>
+      </c>
+      <c r="D95" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="E95" s="20">
         <f>IF($B95="","",INDEX(Simulador!$D$7:$D$232,MATCH($B95,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>116</v>
       </c>
       <c r="F95" s="20"/>
-      <c r="G95" s="13" t="str">
+      <c r="G95" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>116</v>
       </c>
       <c r="H95" s="8" t="str">
         <f>IF($B95="","",INDEX(Simulador!$B$7:$B$232,MATCH($B95,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I95" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I95" s="13">
         <f>IF(OR(H95="",$D95=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D95,Ref_Frete!$A$2:$A$54,0),IF(H95="Pequenos",2,IF(H95="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J95" s="20"/>
-      <c r="K95" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J95" s="20">
+        <v>11.7</v>
+      </c>
+      <c r="K95" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L95" s="13" t="str">
+        <v>19.02</v>
+      </c>
+      <c r="L95" s="13">
         <f>IF(OR($B95="",$C95=""),"",$C95*INDEX(Simulador!$F$7:$F$232,MATCH($B95,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M95" s="13" t="str">
+        <v>54.47</v>
+      </c>
+      <c r="M95" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N95" s="35" t="str">
+        <v>11.600000000000001</v>
+      </c>
+      <c r="N95" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O95" s="12" t="str">
+        <v>44.110000000000021</v>
+      </c>
+      <c r="O95" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.38025862068965532</v>
       </c>
       <c r="P95" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q95" s="19"/>
       <c r="R95" s="19"/>
@@ -22383,27 +22393,27 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>35340.440000000024</v>
+        <v>35456.440000000024</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>5377.2600000000029</v>
+        <v>5396.2800000000034</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>18387.500000000004</v>
+        <v>18441.970000000005</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>3534.0439999999994</v>
+        <v>3545.6439999999993</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>8991.6860000000015</v>
+        <v>9035.7960000000021</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25443050510972687</v>
+        <v>0.25484216689549194</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
[19/10] Mestra: Origem 93 Ads / 94 Organico e STATUS 95 lancados pelo LEO
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2105" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2108" uniqueCount="583">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -2044,7 +2044,21 @@
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -21659,7 +21673,9 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q93" s="19"/>
-      <c r="R93" s="19"/>
+      <c r="R93" s="19" t="s">
+        <v>210</v>
+      </c>
       <c r="S93" t="s">
         <v>558</v>
       </c>
@@ -21722,7 +21738,9 @@
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q94" s="19"/>
-      <c r="R94" s="19"/>
+      <c r="R94" s="19" t="s">
+        <v>207</v>
+      </c>
       <c r="S94" t="s">
         <v>558</v>
       </c>
@@ -21786,6 +21804,9 @@
       </c>
       <c r="Q95" s="19"/>
       <c r="R95" s="19"/>
+      <c r="S95" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="96" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="32"/>
@@ -22420,11 +22441,11 @@
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S94">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+  <conditionalFormatting sqref="S6:S95">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"VÁLIDO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[20/10] Mestra: vendas de 19/10 (L1618-A PR Capital, P3050 BA Interior) nas linhas 96-97; Origem 95-97 fica para a O8
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2108" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2114" uniqueCount="583">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -21809,106 +21809,132 @@
       </c>
     </row>
     <row r="96" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="32"/>
-      <c r="B96" s="19"/>
-      <c r="C96" s="19"/>
-      <c r="D96" s="19"/>
-      <c r="E96" s="20" t="str">
+      <c r="A96" s="32">
+        <v>46314</v>
+      </c>
+      <c r="B96" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="C96" s="19">
+        <v>1</v>
+      </c>
+      <c r="D96" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E96" s="20">
         <f>IF($B96="","",INDEX(Simulador!$D$7:$D$232,MATCH($B96,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>104.9</v>
       </c>
       <c r="F96" s="20"/>
-      <c r="G96" s="13" t="str">
+      <c r="G96" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>104.9</v>
       </c>
       <c r="H96" s="8" t="str">
         <f>IF($B96="","",INDEX(Simulador!$B$7:$B$232,MATCH($B96,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I96" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I96" s="13">
         <f>IF(OR(H96="",$D96=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D96,Ref_Frete!$A$2:$A$54,0),IF(H96="Pequenos",2,IF(H96="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J96" s="20"/>
-      <c r="K96" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J96" s="20">
+        <v>14.22</v>
+      </c>
+      <c r="K96" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L96" s="13" t="str">
+        <v>17.52</v>
+      </c>
+      <c r="L96" s="13">
         <f>IF(OR($B96="",$C96=""),"",$C96*INDEX(Simulador!$F$7:$F$232,MATCH($B96,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M96" s="13" t="str">
+        <v>48.18</v>
+      </c>
+      <c r="M96" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N96" s="35" t="str">
+        <v>10.490000000000002</v>
+      </c>
+      <c r="N96" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O96" s="12" t="str">
+        <v>39.390000000000015</v>
+      </c>
+      <c r="O96" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.37550047664442338</v>
       </c>
       <c r="P96" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q96" s="19"/>
       <c r="R96" s="19"/>
-    </row>
-    <row r="97" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="32"/>
-      <c r="B97" s="19"/>
-      <c r="C97" s="19"/>
-      <c r="D97" s="19"/>
-      <c r="E97" s="20" t="str">
+      <c r="S96" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="97" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="32">
+        <v>46314</v>
+      </c>
+      <c r="B97" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="C97" s="19">
+        <v>1</v>
+      </c>
+      <c r="D97" s="19" t="s">
+        <v>394</v>
+      </c>
+      <c r="E97" s="20">
         <f>IF($B97="","",INDEX(Simulador!$D$7:$D$232,MATCH($B97,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>467.67</v>
       </c>
       <c r="F97" s="20"/>
-      <c r="G97" s="13" t="str">
+      <c r="G97" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>467.67</v>
       </c>
       <c r="H97" s="8" t="str">
         <f>IF($B97="","",INDEX(Simulador!$B$7:$B$232,MATCH($B97,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I97" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I97" s="13">
         <f>IF(OR(H97="",$D97=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D97,Ref_Frete!$A$2:$A$54,0),IF(H97="Pequenos",2,IF(H97="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J97" s="20"/>
-      <c r="K97" s="20" t="str">
+        <v>142</v>
+      </c>
+      <c r="J97" s="20">
+        <v>96.04</v>
+      </c>
+      <c r="K97" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L97" s="13" t="str">
+        <v>82.31</v>
+      </c>
+      <c r="L97" s="13">
         <f>IF(OR($B97="",$C97=""),"",$C97*INDEX(Simulador!$F$7:$F$232,MATCH($B97,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M97" s="13" t="str">
+        <v>240.55</v>
+      </c>
+      <c r="M97" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N97" s="35" t="str">
+        <v>46.767000000000003</v>
+      </c>
+      <c r="N97" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O97" s="12" t="str">
+        <v>144.0030000000001</v>
+      </c>
+      <c r="O97" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.30791583809096179</v>
       </c>
       <c r="P97" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q97" s="19"/>
       <c r="R97" s="19"/>
-    </row>
-    <row r="98" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S97" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="98" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="32"/>
       <c r="B98" s="19"/>
       <c r="C98" s="19"/>
@@ -21958,7 +21984,7 @@
       <c r="Q98" s="19"/>
       <c r="R98" s="19"/>
     </row>
-    <row r="99" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="32"/>
       <c r="B99" s="19"/>
       <c r="C99" s="19"/>
@@ -22008,7 +22034,7 @@
       <c r="Q99" s="19"/>
       <c r="R99" s="19"/>
     </row>
-    <row r="100" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="32"/>
       <c r="B100" s="19"/>
       <c r="C100" s="19"/>
@@ -22058,7 +22084,7 @@
       <c r="Q100" s="19"/>
       <c r="R100" s="19"/>
     </row>
-    <row r="101" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="32"/>
       <c r="B101" s="19"/>
       <c r="C101" s="19"/>
@@ -22108,7 +22134,7 @@
       <c r="Q101" s="19"/>
       <c r="R101" s="19"/>
     </row>
-    <row r="102" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="32"/>
       <c r="B102" s="19"/>
       <c r="C102" s="19"/>
@@ -22158,7 +22184,7 @@
       <c r="Q102" s="19"/>
       <c r="R102" s="19"/>
     </row>
-    <row r="103" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="32"/>
       <c r="B103" s="19"/>
       <c r="C103" s="19"/>
@@ -22208,7 +22234,7 @@
       <c r="Q103" s="19"/>
       <c r="R103" s="19"/>
     </row>
-    <row r="104" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="32"/>
       <c r="B104" s="19"/>
       <c r="C104" s="19"/>
@@ -22258,7 +22284,7 @@
       <c r="Q104" s="19"/>
       <c r="R104" s="19"/>
     </row>
-    <row r="105" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="32"/>
       <c r="B105" s="19"/>
       <c r="C105" s="19"/>
@@ -22308,7 +22334,7 @@
       <c r="Q105" s="19"/>
       <c r="R105" s="19"/>
     </row>
-    <row r="106" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="32"/>
       <c r="B106" s="19"/>
       <c r="C106" s="19"/>
@@ -22358,7 +22384,7 @@
       <c r="Q106" s="19"/>
       <c r="R106" s="19"/>
     </row>
-    <row r="107" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="32"/>
       <c r="B107" s="19"/>
       <c r="C107" s="19"/>
@@ -22408,40 +22434,40 @@
       <c r="Q107" s="19"/>
       <c r="R107" s="19"/>
     </row>
-    <row r="108" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
         <v>249</v>
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>35456.440000000024</v>
+        <v>36029.010000000024</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>5396.2800000000034</v>
+        <v>5496.1100000000042</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>18441.970000000005</v>
+        <v>18730.700000000004</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>3545.6439999999993</v>
+        <v>3602.9009999999989</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>9035.7960000000021</v>
+        <v>9219.1890000000021</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25484216689549194</v>
+        <v>0.25588238477826608</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S95">
+  <conditionalFormatting sqref="S6:S97">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>

</xml_diff>

<commit_message>
[21/10] Mestra: venda de 21/10 (P3070, SP Capital) na linha 98; Origem 95-98 fica para a O8
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2114" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2117" uniqueCount="583">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -21935,54 +21935,67 @@
       </c>
     </row>
     <row r="98" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="32"/>
-      <c r="B98" s="19"/>
-      <c r="C98" s="19"/>
-      <c r="D98" s="19"/>
-      <c r="E98" s="20" t="str">
+      <c r="A98" s="32">
+        <v>46316</v>
+      </c>
+      <c r="B98" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C98" s="19">
+        <v>1</v>
+      </c>
+      <c r="D98" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="E98" s="20">
         <f>IF($B98="","",INDEX(Simulador!$D$7:$D$232,MATCH($B98,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>616.17999999999995</v>
       </c>
       <c r="F98" s="20"/>
-      <c r="G98" s="13" t="str">
+      <c r="G98" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>616.17999999999995</v>
       </c>
       <c r="H98" s="8" t="str">
         <f>IF($B98="","",INDEX(Simulador!$B$7:$B$232,MATCH($B98,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I98" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I98" s="13">
         <f>IF(OR(H98="",$D98=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D98,Ref_Frete!$A$2:$A$54,0),IF(H98="Pequenos",2,IF(H98="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J98" s="20"/>
-      <c r="K98" s="20" t="str">
+        <v>34.9</v>
+      </c>
+      <c r="J98" s="20">
+        <v>30.29</v>
+      </c>
+      <c r="K98" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L98" s="13" t="str">
+        <v>87.9</v>
+      </c>
+      <c r="L98" s="13">
         <f>IF(OR($B98="",$C98=""),"",$C98*INDEX(Simulador!$F$7:$F$232,MATCH($B98,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M98" s="13" t="str">
+        <v>307.26</v>
+      </c>
+      <c r="M98" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N98" s="35" t="str">
+        <v>61.617999999999995</v>
+      </c>
+      <c r="N98" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O98" s="12" t="str">
+        <v>164.012</v>
+      </c>
+      <c r="O98" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.26617546820734206</v>
       </c>
       <c r="P98" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q98" s="19"/>
       <c r="R98" s="19"/>
+      <c r="S98" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="99" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="32"/>
@@ -22440,34 +22453,34 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>36029.010000000024</v>
+        <v>36645.190000000024</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>5496.1100000000042</v>
+        <v>5584.0100000000039</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>18730.700000000004</v>
+        <v>19037.960000000003</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>3602.9009999999989</v>
+        <v>3664.5189999999989</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>9219.1890000000021</v>
+        <v>9383.2010000000028</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25588238477826608</v>
+        <v>0.25605546048471839</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S97">
+  <conditionalFormatting sqref="S6:S98">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>

</xml_diff>

<commit_message>
[22/10] Mestra: vendas de 21/10 (PXP x2, RS, 25,5%) e 22/10 (P3060, ES, 30,7%); totais R$ 37.492,39 / 26%
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_5.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2117" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2123" uniqueCount="583">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -21998,104 +21998,130 @@
       </c>
     </row>
     <row r="99" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="32"/>
-      <c r="B99" s="19"/>
-      <c r="C99" s="19"/>
-      <c r="D99" s="19"/>
-      <c r="E99" s="20" t="str">
+      <c r="A99" s="32">
+        <v>46316</v>
+      </c>
+      <c r="B99" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="C99" s="19">
+        <v>2</v>
+      </c>
+      <c r="D99" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="E99" s="20">
         <f>IF($B99="","",INDEX(Simulador!$D$7:$D$232,MATCH($B99,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>167.89</v>
       </c>
       <c r="F99" s="20"/>
-      <c r="G99" s="13" t="str">
+      <c r="G99" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>335.78</v>
       </c>
       <c r="H99" s="8" t="str">
         <f>IF($B99="","",INDEX(Simulador!$B$7:$B$232,MATCH($B99,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I99" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I99" s="13">
         <f>IF(OR(H99="",$D99=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D99,Ref_Frete!$A$2:$A$54,0),IF(H99="Pequenos",2,IF(H99="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J99" s="20"/>
-      <c r="K99" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J99" s="20">
+        <v>23.1</v>
+      </c>
+      <c r="K99" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L99" s="13" t="str">
+        <v>48.69</v>
+      </c>
+      <c r="L99" s="13">
         <f>IF(OR($B99="",$C99=""),"",$C99*INDEX(Simulador!$F$7:$F$232,MATCH($B99,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M99" s="13" t="str">
+        <v>169.58</v>
+      </c>
+      <c r="M99" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N99" s="35" t="str">
+        <v>33.577999999999996</v>
+      </c>
+      <c r="N99" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O99" s="12" t="str">
+        <v>85.731999999999914</v>
+      </c>
+      <c r="O99" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.25532193698254785</v>
       </c>
       <c r="P99" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q99" s="19"/>
       <c r="R99" s="19"/>
+      <c r="S99" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="100" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="32"/>
-      <c r="B100" s="19"/>
-      <c r="C100" s="19"/>
-      <c r="D100" s="19"/>
-      <c r="E100" s="20" t="str">
+      <c r="A100" s="32">
+        <v>46317</v>
+      </c>
+      <c r="B100" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C100" s="19">
+        <v>1</v>
+      </c>
+      <c r="D100" s="19" t="s">
+        <v>409</v>
+      </c>
+      <c r="E100" s="20">
         <f>IF($B100="","",INDEX(Simulador!$D$7:$D$232,MATCH($B100,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>511.42</v>
       </c>
       <c r="F100" s="20"/>
-      <c r="G100" s="13" t="str">
+      <c r="G100" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>511.42</v>
       </c>
       <c r="H100" s="8" t="str">
         <f>IF($B100="","",INDEX(Simulador!$B$7:$B$232,MATCH($B100,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I100" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I100" s="13">
         <f>IF(OR(H100="",$D100=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D100,Ref_Frete!$A$2:$A$54,0),IF(H100="Pequenos",2,IF(H100="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J100" s="20"/>
-      <c r="K100" s="20" t="str">
+        <v>59.9</v>
+      </c>
+      <c r="J100" s="20">
+        <v>43.63</v>
+      </c>
+      <c r="K100" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L100" s="13" t="str">
+        <v>77.13</v>
+      </c>
+      <c r="L100" s="13">
         <f>IF(OR($B100="",$C100=""),"",$C100*INDEX(Simulador!$F$7:$F$232,MATCH($B100,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M100" s="13" t="str">
+        <v>242.26</v>
+      </c>
+      <c r="M100" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N100" s="35" t="str">
+        <v>51.142000000000003</v>
+      </c>
+      <c r="N100" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O100" s="12" t="str">
+        <v>157.15800000000007</v>
+      </c>
+      <c r="O100" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.30729732900551421</v>
       </c>
       <c r="P100" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q100" s="19"/>
       <c r="R100" s="19"/>
+      <c r="S100" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="101" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="32"/>
@@ -22453,34 +22479,34 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>36645.190000000024</v>
+        <v>37492.390000000021</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>5584.0100000000039</v>
+        <v>5709.8300000000036</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>19037.960000000003</v>
+        <v>19449.800000000003</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>3664.5189999999989</v>
+        <v>3749.2389999999987</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>9383.2010000000028</v>
+        <v>9626.0910000000022</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25605546048471839</v>
+        <v>0.25674786269960376</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S98">
+  <conditionalFormatting sqref="S6:S100">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>

</xml_diff>